<commit_message>
changed user choosing steady state to graph, added cool cursor featrure to see detialed data point values
</commit_message>
<xml_diff>
--- a/NURBS IDX30 PYTHON ANALYSIS/Back_final_15_2_26/15gps/5mps_analysis.xlsx
+++ b/NURBS IDX30 PYTHON ANALYSIS/Back_final_15_2_26/15gps/5mps_analysis.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>Time</t>
   </si>
@@ -79,13 +79,34 @@
     <t>Q</t>
   </si>
   <si>
-    <t>rolling_std</t>
-  </si>
-  <si>
     <t>steady_state</t>
   </si>
   <si>
-    <t>avg_Q_steady</t>
+    <t>Averages</t>
+  </si>
+  <si>
+    <t>RTD_OUT_unc</t>
+  </si>
+  <si>
+    <t>RTD_IN_unc</t>
+  </si>
+  <si>
+    <t>RTD_unc</t>
+  </si>
+  <si>
+    <t>Delta_RTD</t>
+  </si>
+  <si>
+    <t>Rel_unc</t>
+  </si>
+  <si>
+    <t>ABS_unc</t>
+  </si>
+  <si>
+    <t>Average Q (W)</t>
+  </si>
+  <si>
+    <t>Average Q Uncertainty (W)</t>
   </si>
 </sst>
 </file>
@@ -421,10 +442,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X36"/>
+  <dimension ref="A1:AC36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:24">
+    <row r="1" spans="1:29">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -497,8 +518,23 @@
       <c r="X1" t="s">
         <v>23</v>
       </c>
+      <c r="Y1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>28</v>
+      </c>
     </row>
-    <row r="2" spans="1:24">
+    <row r="2" spans="1:29">
       <c r="A2" s="1">
         <v>46068.56060113426</v>
       </c>
@@ -562,14 +598,32 @@
       <c r="U2">
         <v>635.007891149283</v>
       </c>
-      <c r="W2" t="b">
+      <c r="V2" t="b">
         <v>0</v>
       </c>
+      <c r="W2" t="s">
+        <v>29</v>
+      </c>
       <c r="X2">
-        <v>642.5360960986419</v>
+        <v>0.24194208</v>
+      </c>
+      <c r="Y2">
+        <v>0.26116995</v>
+      </c>
+      <c r="Z2">
+        <v>0.3560136413927547</v>
+      </c>
+      <c r="AA2">
+        <v>9.613934999999998</v>
+      </c>
+      <c r="AB2">
+        <v>0.03835746435821478</v>
+      </c>
+      <c r="AC2">
+        <v>24.35729255194375</v>
       </c>
     </row>
-    <row r="3" spans="1:24">
+    <row r="3" spans="1:29">
       <c r="A3" s="1">
         <v>46068.560716875</v>
       </c>
@@ -633,11 +687,32 @@
       <c r="U3">
         <v>636.859153134169</v>
       </c>
-      <c r="W3" t="b">
+      <c r="V3" t="b">
         <v>0</v>
       </c>
+      <c r="W3">
+        <v>642.365926539937</v>
+      </c>
+      <c r="X3">
+        <v>0.241916376</v>
+      </c>
+      <c r="Y3">
+        <v>0.26117918</v>
+      </c>
+      <c r="Z3">
+        <v>0.3560029452721505</v>
+      </c>
+      <c r="AA3">
+        <v>9.631402000000001</v>
+      </c>
+      <c r="AB3">
+        <v>0.03829156130452172</v>
+      </c>
+      <c r="AC3">
+        <v>24.38633130458282</v>
+      </c>
     </row>
-    <row r="4" spans="1:24">
+    <row r="4" spans="1:29">
       <c r="A4" s="1">
         <v>46068.56083319445</v>
       </c>
@@ -701,14 +776,32 @@
       <c r="U4">
         <v>637.1740984334546</v>
       </c>
-      <c r="V4">
-        <v>1.170385654120398</v>
-      </c>
-      <c r="W4" t="b">
-        <v>1</v>
+      <c r="V4" t="b">
+        <v>0</v>
+      </c>
+      <c r="W4" t="s">
+        <v>30</v>
+      </c>
+      <c r="X4">
+        <v>0.241910346</v>
+      </c>
+      <c r="Y4">
+        <v>0.261177588</v>
+      </c>
+      <c r="Z4">
+        <v>0.3559976797330812</v>
+      </c>
+      <c r="AA4">
+        <v>9.633620999999998</v>
+      </c>
+      <c r="AB4">
+        <v>0.03828281526092951</v>
+      </c>
+      <c r="AC4">
+        <v>24.39281829937726</v>
       </c>
     </row>
-    <row r="5" spans="1:24">
+    <row r="5" spans="1:29">
       <c r="A5" s="1">
         <v>46068.56094951389</v>
       </c>
@@ -772,14 +865,32 @@
       <c r="U5">
         <v>633.429524269103</v>
       </c>
-      <c r="V5">
-        <v>2.07699223100638</v>
-      </c>
-      <c r="W5" t="b">
-        <v>1</v>
+      <c r="V5" t="b">
+        <v>0</v>
+      </c>
+      <c r="W5">
+        <v>24.47006440626338</v>
+      </c>
+      <c r="X5">
+        <v>0.24190051</v>
+      </c>
+      <c r="Y5">
+        <v>0.261180134</v>
+      </c>
+      <c r="Z5">
+        <v>0.3559928638814521</v>
+      </c>
+      <c r="AA5">
+        <v>9.639811999999999</v>
+      </c>
+      <c r="AB5">
+        <v>0.03825942468394949</v>
+      </c>
+      <c r="AC5">
+        <v>24.2346491763637</v>
       </c>
     </row>
-    <row r="6" spans="1:24">
+    <row r="6" spans="1:29">
       <c r="A6" s="1">
         <v>46068.56106525463</v>
       </c>
@@ -843,14 +954,29 @@
       <c r="U6">
         <v>639.2553770869982</v>
       </c>
-      <c r="V6">
-        <v>2.952234113396289</v>
-      </c>
-      <c r="W6" t="b">
+      <c r="V6" t="b">
         <v>1</v>
       </c>
+      <c r="X6">
+        <v>0.24187671</v>
+      </c>
+      <c r="Y6">
+        <v>0.261180452</v>
+      </c>
+      <c r="Z6">
+        <v>0.3559769253018353</v>
+      </c>
+      <c r="AA6">
+        <v>9.651871</v>
+      </c>
+      <c r="AB6">
+        <v>0.03821329723524135</v>
+      </c>
+      <c r="AC6">
+        <v>24.42805573385176</v>
+      </c>
     </row>
-    <row r="7" spans="1:24">
+    <row r="7" spans="1:29">
       <c r="A7" s="1">
         <v>46068.56118157408</v>
       </c>
@@ -914,14 +1040,29 @@
       <c r="U7">
         <v>645.5955693679837</v>
       </c>
-      <c r="V7">
-        <v>6.084834324828289</v>
-      </c>
-      <c r="W7" t="b">
-        <v>0</v>
+      <c r="V7" t="b">
+        <v>1</v>
+      </c>
+      <c r="X7">
+        <v>0.241817052</v>
+      </c>
+      <c r="Y7">
+        <v>0.261180134</v>
+      </c>
+      <c r="Z7">
+        <v>0.3559361586495936</v>
+      </c>
+      <c r="AA7">
+        <v>9.681540999999996</v>
+      </c>
+      <c r="AB7">
+        <v>0.03810015699911633</v>
+      </c>
+      <c r="AC7">
+        <v>24.59729255085407</v>
       </c>
     </row>
-    <row r="8" spans="1:24">
+    <row r="8" spans="1:29">
       <c r="A8" s="1">
         <v>46068.56129731482</v>
       </c>
@@ -985,14 +1126,29 @@
       <c r="U8">
         <v>642.0941663253152</v>
       </c>
-      <c r="V8">
-        <v>3.175861714209091</v>
-      </c>
-      <c r="W8" t="b">
-        <v>0</v>
+      <c r="V8" t="b">
+        <v>1</v>
+      </c>
+      <c r="X8">
+        <v>0.241780242</v>
+      </c>
+      <c r="Y8">
+        <v>0.261176316</v>
+      </c>
+      <c r="Z8">
+        <v>0.355908349804989</v>
+      </c>
+      <c r="AA8">
+        <v>9.698036999999999</v>
+      </c>
+      <c r="AB8">
+        <v>0.0380370514329286</v>
+      </c>
+      <c r="AC8">
+        <v>24.42336882929943</v>
       </c>
     </row>
-    <row r="9" spans="1:24">
+    <row r="9" spans="1:29">
       <c r="A9" s="1">
         <v>46068.56141363426</v>
       </c>
@@ -1056,14 +1212,29 @@
       <c r="U9">
         <v>645.7356518243965</v>
       </c>
-      <c r="V9">
-        <v>2.063163549900994</v>
-      </c>
-      <c r="W9" t="b">
+      <c r="V9" t="b">
         <v>1</v>
       </c>
+      <c r="X9">
+        <v>0.24175676</v>
+      </c>
+      <c r="Y9">
+        <v>0.261161994</v>
+      </c>
+      <c r="Z9">
+        <v>0.3558818878725829</v>
+      </c>
+      <c r="AA9">
+        <v>9.702617000000004</v>
+      </c>
+      <c r="AB9">
+        <v>0.03801770651489158</v>
+      </c>
+      <c r="AC9">
+        <v>24.54938849726212</v>
+      </c>
     </row>
-    <row r="10" spans="1:24">
+    <row r="10" spans="1:29">
       <c r="A10" s="1">
         <v>46068.561529375</v>
       </c>
@@ -1127,14 +1298,29 @@
       <c r="U10">
         <v>638.051283177792</v>
       </c>
-      <c r="V10">
-        <v>3.843931196953672</v>
-      </c>
-      <c r="W10" t="b">
-        <v>0</v>
+      <c r="V10" t="b">
+        <v>1</v>
+      </c>
+      <c r="X10">
+        <v>0.241804676</v>
+      </c>
+      <c r="Y10">
+        <v>0.261152446</v>
+      </c>
+      <c r="Z10">
+        <v>0.3559074337341774</v>
+      </c>
+      <c r="AA10">
+        <v>9.673884999999999</v>
+      </c>
+      <c r="AB10">
+        <v>0.03812536801905542</v>
+      </c>
+      <c r="AC10">
+        <v>24.32593998618387</v>
       </c>
     </row>
-    <row r="11" spans="1:24">
+    <row r="11" spans="1:29">
       <c r="A11" s="1">
         <v>46068.56164511574</v>
       </c>
@@ -1198,14 +1384,29 @@
       <c r="U11">
         <v>645.4102079647308</v>
       </c>
-      <c r="V11">
-        <v>4.3456723534752</v>
-      </c>
-      <c r="W11" t="b">
-        <v>0</v>
+      <c r="V11" t="b">
+        <v>1</v>
+      </c>
+      <c r="X11">
+        <v>0.241791348</v>
+      </c>
+      <c r="Y11">
+        <v>0.26115531</v>
+      </c>
+      <c r="Z11">
+        <v>0.3559004803436674</v>
+      </c>
+      <c r="AA11">
+        <v>9.681981</v>
+      </c>
+      <c r="AB11">
+        <v>0.03809498900355612</v>
+      </c>
+      <c r="AC11">
+        <v>24.58689477519929</v>
       </c>
     </row>
-    <row r="12" spans="1:24">
+    <row r="12" spans="1:29">
       <c r="A12" s="1">
         <v>46068.56176143519</v>
       </c>
@@ -1269,14 +1470,29 @@
       <c r="U12">
         <v>643.4669427018275</v>
       </c>
-      <c r="V12">
-        <v>3.813559622848506</v>
-      </c>
-      <c r="W12" t="b">
-        <v>0</v>
+      <c r="V12" t="b">
+        <v>1</v>
+      </c>
+      <c r="X12">
+        <v>0.241798012</v>
+      </c>
+      <c r="Y12">
+        <v>0.261145444</v>
+      </c>
+      <c r="Z12">
+        <v>0.3558977683677003</v>
+      </c>
+      <c r="AA12">
+        <v>9.673715999999999</v>
+      </c>
+      <c r="AB12">
+        <v>0.03812502409199905</v>
+      </c>
+      <c r="AC12">
+        <v>24.53219269291214</v>
       </c>
     </row>
-    <row r="13" spans="1:24">
+    <row r="13" spans="1:29">
       <c r="A13" s="1">
         <v>46068.56187717593</v>
       </c>
@@ -1340,14 +1556,29 @@
       <c r="U13">
         <v>640.4862750844075</v>
       </c>
-      <c r="V13">
-        <v>2.480113382404472</v>
-      </c>
-      <c r="W13" t="b">
+      <c r="V13" t="b">
         <v>1</v>
       </c>
+      <c r="X13">
+        <v>0.241802772</v>
+      </c>
+      <c r="Y13">
+        <v>0.261136214</v>
+      </c>
+      <c r="Z13">
+        <v>0.3558942298059042</v>
+      </c>
+      <c r="AA13">
+        <v>9.666720999999995</v>
+      </c>
+      <c r="AB13">
+        <v>0.03815036136552507</v>
+      </c>
+      <c r="AC13">
+        <v>24.43478284412924</v>
+      </c>
     </row>
-    <row r="14" spans="1:24">
+    <row r="14" spans="1:29">
       <c r="A14" s="1">
         <v>46068.56199349537</v>
       </c>
@@ -1411,14 +1642,29 @@
       <c r="U14">
         <v>643.8171150619287</v>
       </c>
-      <c r="V14">
-        <v>1.830368591440265</v>
-      </c>
-      <c r="W14" t="b">
+      <c r="V14" t="b">
         <v>1</v>
       </c>
+      <c r="X14">
+        <v>0.241797694</v>
+      </c>
+      <c r="Y14">
+        <v>0.261128256</v>
+      </c>
+      <c r="Z14">
+        <v>0.3558849405430345</v>
+      </c>
+      <c r="AA14">
+        <v>9.665280999999993</v>
+      </c>
+      <c r="AB14">
+        <v>0.03815472727020246</v>
+      </c>
+      <c r="AC14">
+        <v>24.56466643707644</v>
+      </c>
     </row>
-    <row r="15" spans="1:24">
+    <row r="15" spans="1:29">
       <c r="A15" s="1">
         <v>46068.56210923611</v>
       </c>
@@ -1482,14 +1728,29 @@
       <c r="U15">
         <v>640.920259413961</v>
       </c>
-      <c r="V15">
-        <v>1.810828999810574</v>
-      </c>
-      <c r="W15" t="b">
+      <c r="V15" t="b">
         <v>1</v>
       </c>
+      <c r="X15">
+        <v>0.24179357</v>
+      </c>
+      <c r="Y15">
+        <v>0.261119026</v>
+      </c>
+      <c r="Z15">
+        <v>0.3558753661501926</v>
+      </c>
+      <c r="AA15">
+        <v>9.662728000000001</v>
+      </c>
+      <c r="AB15">
+        <v>0.03816315954765462</v>
+      </c>
+      <c r="AC15">
+        <v>24.45954211733918</v>
+      </c>
     </row>
-    <row r="16" spans="1:24">
+    <row r="16" spans="1:29">
       <c r="A16" s="1">
         <v>46068.56222555556</v>
       </c>
@@ -1553,14 +1814,29 @@
       <c r="U16">
         <v>643.3438372566179</v>
       </c>
-      <c r="V16">
-        <v>1.553999897340002</v>
-      </c>
-      <c r="W16" t="b">
+      <c r="V16" t="b">
         <v>1</v>
       </c>
+      <c r="X16">
+        <v>0.241779608</v>
+      </c>
+      <c r="Y16">
+        <v>0.261115526</v>
+      </c>
+      <c r="Z16">
+        <v>0.3558633119090676</v>
+      </c>
+      <c r="AA16">
+        <v>9.667959000000003</v>
+      </c>
+      <c r="AB16">
+        <v>0.03814272568945068</v>
+      </c>
+      <c r="AC16">
+        <v>24.53888750847778</v>
+      </c>
     </row>
-    <row r="17" spans="1:23">
+    <row r="17" spans="1:29">
       <c r="A17" s="1">
         <v>46068.562341875</v>
       </c>
@@ -1624,14 +1900,29 @@
       <c r="U17">
         <v>640.7224724921551</v>
       </c>
-      <c r="V17">
-        <v>1.459703306282813</v>
-      </c>
-      <c r="W17" t="b">
+      <c r="V17" t="b">
         <v>1</v>
       </c>
+      <c r="X17">
+        <v>0.241786906</v>
+      </c>
+      <c r="Y17">
+        <v>0.2611238</v>
+      </c>
+      <c r="Z17">
+        <v>0.355874341361516</v>
+      </c>
+      <c r="AA17">
+        <v>9.668447</v>
+      </c>
+      <c r="AB17">
+        <v>0.03814203368699726</v>
+      </c>
+      <c r="AC17">
+        <v>24.43845812981196</v>
+      </c>
     </row>
-    <row r="18" spans="1:23">
+    <row r="18" spans="1:29">
       <c r="A18" s="1">
         <v>46068.56245761574</v>
       </c>
@@ -1695,14 +1986,29 @@
       <c r="U18">
         <v>638.7948352043771</v>
       </c>
-      <c r="V18">
-        <v>2.283300185145247</v>
-      </c>
-      <c r="W18" t="b">
+      <c r="V18" t="b">
         <v>1</v>
       </c>
+      <c r="X18">
+        <v>0.241797378</v>
+      </c>
+      <c r="Y18">
+        <v>0.261106614</v>
+      </c>
+      <c r="Z18">
+        <v>0.3558688464620356</v>
+      </c>
+      <c r="AA18">
+        <v>9.654617999999999</v>
+      </c>
+      <c r="AB18">
+        <v>0.03819236509747999</v>
+      </c>
+      <c r="AC18">
+        <v>24.39708556851014</v>
+      </c>
     </row>
-    <row r="19" spans="1:23">
+    <row r="19" spans="1:29">
       <c r="A19" s="1">
         <v>46068.56257393518</v>
       </c>
@@ -1766,14 +2072,29 @@
       <c r="U19">
         <v>641.8978039057973</v>
       </c>
-      <c r="V19">
-        <v>1.56661015184247</v>
-      </c>
-      <c r="W19" t="b">
+      <c r="V19" t="b">
         <v>1</v>
       </c>
+      <c r="X19">
+        <v>0.241790078</v>
+      </c>
+      <c r="Y19">
+        <v>0.261089428</v>
+      </c>
+      <c r="Z19">
+        <v>0.355851276845557</v>
+      </c>
+      <c r="AA19">
+        <v>9.649675000000002</v>
+      </c>
+      <c r="AB19">
+        <v>0.03820883076411563</v>
+      </c>
+      <c r="AC19">
+        <v>24.52616455729409</v>
+      </c>
     </row>
-    <row r="20" spans="1:23">
+    <row r="20" spans="1:29">
       <c r="A20" s="1">
         <v>46068.56268967593</v>
       </c>
@@ -1837,14 +2158,29 @@
       <c r="U20">
         <v>641.5720019770681</v>
       </c>
-      <c r="V20">
-        <v>1.705247633146532</v>
-      </c>
-      <c r="W20" t="b">
+      <c r="V20" t="b">
         <v>1</v>
       </c>
+      <c r="X20">
+        <v>0.2417685</v>
+      </c>
+      <c r="Y20">
+        <v>0.26108338</v>
+      </c>
+      <c r="Z20">
+        <v>0.3558321780059729</v>
+      </c>
+      <c r="AA20">
+        <v>9.657440000000001</v>
+      </c>
+      <c r="AB20">
+        <v>0.03817830574849729</v>
+      </c>
+      <c r="AC20">
+        <v>24.49413205115602</v>
+      </c>
     </row>
-    <row r="21" spans="1:23">
+    <row r="21" spans="1:29">
       <c r="A21" s="1">
         <v>46068.56280541667</v>
       </c>
@@ -1908,14 +2244,29 @@
       <c r="U21">
         <v>642.8010032046559</v>
       </c>
-      <c r="V21">
-        <v>0.6367050452194546</v>
-      </c>
-      <c r="W21" t="b">
+      <c r="V21" t="b">
         <v>1</v>
       </c>
+      <c r="X21">
+        <v>0.241755174</v>
+      </c>
+      <c r="Y21">
+        <v>0.261085926</v>
+      </c>
+      <c r="Z21">
+        <v>0.3558249919708392</v>
+      </c>
+      <c r="AA21">
+        <v>9.665376000000002</v>
+      </c>
+      <c r="AB21">
+        <v>0.03814839246209575</v>
+      </c>
+      <c r="AC21">
+        <v>24.52182494528008</v>
+      </c>
     </row>
-    <row r="22" spans="1:23">
+    <row r="22" spans="1:29">
       <c r="A22" s="1">
         <v>46068.56292173611</v>
       </c>
@@ -1979,14 +2330,29 @@
       <c r="U22">
         <v>638.3833113770795</v>
       </c>
-      <c r="V22">
-        <v>2.280138623100127</v>
-      </c>
-      <c r="W22" t="b">
+      <c r="V22" t="b">
         <v>1</v>
       </c>
+      <c r="X22">
+        <v>0.241762154</v>
+      </c>
+      <c r="Y22">
+        <v>0.261096748</v>
+      </c>
+      <c r="Z22">
+        <v>0.3558376749627493</v>
+      </c>
+      <c r="AA22">
+        <v>9.667297000000005</v>
+      </c>
+      <c r="AB22">
+        <v>0.03814259894364048</v>
+      </c>
+      <c r="AC22">
+        <v>24.3495986181691</v>
+      </c>
     </row>
-    <row r="23" spans="1:23">
+    <row r="23" spans="1:29">
       <c r="A23" s="1">
         <v>46068.56303805555</v>
       </c>
@@ -2050,14 +2416,29 @@
       <c r="U23">
         <v>642.4080030307586</v>
       </c>
-      <c r="V23">
-        <v>2.445015103134204</v>
-      </c>
-      <c r="W23" t="b">
+      <c r="V23" t="b">
         <v>1</v>
       </c>
+      <c r="X23">
+        <v>0.24174724</v>
+      </c>
+      <c r="Y23">
+        <v>0.26108147</v>
+      </c>
+      <c r="Z23">
+        <v>0.3558163318693768</v>
+      </c>
+      <c r="AA23">
+        <v>9.667114999999995</v>
+      </c>
+      <c r="AB23">
+        <v>0.03814113711054861</v>
+      </c>
+      <c r="AC23">
+        <v>24.50217172450989</v>
+      </c>
     </row>
-    <row r="24" spans="1:23">
+    <row r="24" spans="1:29">
       <c r="A24" s="1">
         <v>46068.5631537963</v>
       </c>
@@ -2121,14 +2502,29 @@
       <c r="U24">
         <v>643.2032508663279</v>
       </c>
-      <c r="V24">
-        <v>2.584001377295857</v>
-      </c>
-      <c r="W24" t="b">
+      <c r="V24" t="b">
         <v>1</v>
       </c>
+      <c r="X24">
+        <v>0.241756442</v>
+      </c>
+      <c r="Y24">
+        <v>0.26108179</v>
+      </c>
+      <c r="Z24">
+        <v>0.355822818714741</v>
+      </c>
+      <c r="AA24">
+        <v>9.662673999999996</v>
+      </c>
+      <c r="AB24">
+        <v>0.03815811003209012</v>
+      </c>
+      <c r="AC24">
+        <v>24.54342041955541</v>
+      </c>
     </row>
-    <row r="25" spans="1:23">
+    <row r="25" spans="1:29">
       <c r="A25" s="1">
         <v>46068.56327011574</v>
       </c>
@@ -2192,14 +2588,29 @@
       <c r="U25">
         <v>642.7162558321727</v>
       </c>
-      <c r="V25">
-        <v>0.4009578267221894</v>
-      </c>
-      <c r="W25" t="b">
+      <c r="V25" t="b">
         <v>1</v>
       </c>
+      <c r="X25">
+        <v>0.24174851</v>
+      </c>
+      <c r="Y25">
+        <v>0.261079562</v>
+      </c>
+      <c r="Z25">
+        <v>0.355815794732797</v>
+      </c>
+      <c r="AA25">
+        <v>9.665526</v>
+      </c>
+      <c r="AB25">
+        <v>0.0381469228409921</v>
+      </c>
+      <c r="AC25">
+        <v>24.51764741988123</v>
+      </c>
     </row>
-    <row r="26" spans="1:23">
+    <row r="26" spans="1:29">
       <c r="A26" s="1">
         <v>46068.56338585648</v>
       </c>
@@ -2263,14 +2674,29 @@
       <c r="U26">
         <v>638.3165285859485</v>
       </c>
-      <c r="V26">
-        <v>2.691802947531316</v>
-      </c>
-      <c r="W26" t="b">
+      <c r="V26" t="b">
         <v>1</v>
       </c>
+      <c r="X26">
+        <v>0.241740258</v>
+      </c>
+      <c r="Y26">
+        <v>0.261066512</v>
+      </c>
+      <c r="Z26">
+        <v>0.3558006127394284</v>
+      </c>
+      <c r="AA26">
+        <v>9.663127000000003</v>
+      </c>
+      <c r="AB26">
+        <v>0.03815422638410083</v>
+      </c>
+      <c r="AC26">
+        <v>24.35447333638165</v>
+      </c>
     </row>
-    <row r="27" spans="1:23">
+    <row r="27" spans="1:29">
       <c r="A27" s="1">
         <v>46068.56350159722</v>
       </c>
@@ -2334,14 +2760,29 @@
       <c r="U27">
         <v>640.3419811688776</v>
       </c>
-      <c r="V27">
-        <v>2.202167045724217</v>
-      </c>
-      <c r="W27" t="b">
+      <c r="V27" t="b">
         <v>1</v>
       </c>
+      <c r="X27">
+        <v>0.241709162</v>
+      </c>
+      <c r="Y27">
+        <v>0.261071286</v>
+      </c>
+      <c r="Z27">
+        <v>0.3557829891498975</v>
+      </c>
+      <c r="AA27">
+        <v>9.681061999999997</v>
+      </c>
+      <c r="AB27">
+        <v>0.03808664555962978</v>
+      </c>
+      <c r="AC27">
+        <v>24.38847807373017</v>
+      </c>
     </row>
-    <row r="28" spans="1:23">
+    <row r="28" spans="1:29">
       <c r="A28" s="1">
         <v>46068.56361791667</v>
       </c>
@@ -2405,14 +2846,29 @@
       <c r="U28">
         <v>644.2171731840593</v>
       </c>
-      <c r="V28">
-        <v>2.99825443643052</v>
-      </c>
-      <c r="W28" t="b">
+      <c r="V28" t="b">
         <v>1</v>
       </c>
+      <c r="X28">
+        <v>0.241701228</v>
+      </c>
+      <c r="Y28">
+        <v>0.261070014</v>
+      </c>
+      <c r="Z28">
+        <v>0.3557766656579211</v>
+      </c>
+      <c r="AA28">
+        <v>9.684393</v>
+      </c>
+      <c r="AB28">
+        <v>0.03807381864758867</v>
+      </c>
+      <c r="AC28">
+        <v>24.52780782147209</v>
+      </c>
     </row>
-    <row r="29" spans="1:23">
+    <row r="29" spans="1:29">
       <c r="A29" s="1">
         <v>46068.56373423611</v>
       </c>
@@ -2476,14 +2932,29 @@
       <c r="U29">
         <v>645.5715820718979</v>
       </c>
-      <c r="V29">
-        <v>2.714168448311729</v>
-      </c>
-      <c r="W29" t="b">
+      <c r="V29" t="b">
         <v>1</v>
       </c>
+      <c r="X29">
+        <v>0.24164189</v>
+      </c>
+      <c r="Y29">
+        <v>0.261070332</v>
+      </c>
+      <c r="Z29">
+        <v>0.3557365897027776</v>
+      </c>
+      <c r="AA29">
+        <v>9.714220999999995</v>
+      </c>
+      <c r="AB29">
+        <v>0.03796100758470099</v>
+      </c>
+      <c r="AC29">
+        <v>24.50654772349873</v>
+      </c>
     </row>
-    <row r="30" spans="1:23">
+    <row r="30" spans="1:29">
       <c r="A30" s="1">
         <v>46068.56384997685</v>
       </c>
@@ -2547,14 +3018,29 @@
       <c r="U30">
         <v>647.075696837504</v>
       </c>
-      <c r="V30">
-        <v>1.429915040651149</v>
-      </c>
-      <c r="W30" t="b">
+      <c r="V30" t="b">
         <v>1</v>
       </c>
+      <c r="X30">
+        <v>0.241626658</v>
+      </c>
+      <c r="Y30">
+        <v>0.261062374</v>
+      </c>
+      <c r="Z30">
+        <v>0.3557204028092356</v>
+      </c>
+      <c r="AA30">
+        <v>9.717858</v>
+      </c>
+      <c r="AB30">
+        <v>0.03794617958888769</v>
+      </c>
+      <c r="AC30">
+        <v>24.55405059980057</v>
+      </c>
     </row>
-    <row r="31" spans="1:23">
+    <row r="31" spans="1:29">
       <c r="A31" s="1">
         <v>46068.56396571759</v>
       </c>
@@ -2618,14 +3104,29 @@
       <c r="U31">
         <v>639.8552756285068</v>
       </c>
-      <c r="V31">
-        <v>3.809483845575735</v>
-      </c>
-      <c r="W31" t="b">
-        <v>0</v>
+      <c r="V31" t="b">
+        <v>1</v>
+      </c>
+      <c r="X31">
+        <v>0.241648236</v>
+      </c>
+      <c r="Y31">
+        <v>0.261074788</v>
+      </c>
+      <c r="Z31">
+        <v>0.3557441705652485</v>
+      </c>
+      <c r="AA31">
+        <v>9.713276</v>
+      </c>
+      <c r="AB31">
+        <v>0.03796519741951783</v>
+      </c>
+      <c r="AC31">
+        <v>24.29223185915626</v>
       </c>
     </row>
-    <row r="32" spans="1:23">
+    <row r="32" spans="1:29">
       <c r="A32" s="1">
         <v>46068.56408203704</v>
       </c>
@@ -2689,14 +3190,29 @@
       <c r="U32">
         <v>643.0545534872359</v>
       </c>
-      <c r="V32">
-        <v>3.617997952277506</v>
-      </c>
-      <c r="W32" t="b">
-        <v>0</v>
+      <c r="V32" t="b">
+        <v>1</v>
+      </c>
+      <c r="X32">
+        <v>0.24166664</v>
+      </c>
+      <c r="Y32">
+        <v>0.261076378</v>
+      </c>
+      <c r="Z32">
+        <v>0.3557578390401095</v>
+      </c>
+      <c r="AA32">
+        <v>9.704869000000002</v>
+      </c>
+      <c r="AB32">
+        <v>0.0379971633303133</v>
+      </c>
+      <c r="AC32">
+        <v>24.43424889915619</v>
       </c>
     </row>
-    <row r="33" spans="1:23">
+    <row r="33" spans="1:29">
       <c r="A33" s="1">
         <v>46068.56419777778</v>
       </c>
@@ -2760,14 +3276,29 @@
       <c r="U33">
         <v>645.492204458209</v>
       </c>
-      <c r="V33">
-        <v>2.827026933746767</v>
-      </c>
-      <c r="W33" t="b">
+      <c r="V33" t="b">
         <v>1</v>
       </c>
+      <c r="X33">
+        <v>0.24165014</v>
+      </c>
+      <c r="Y33">
+        <v>0.261076378</v>
+      </c>
+      <c r="Z33">
+        <v>0.3557466307804172</v>
+      </c>
+      <c r="AA33">
+        <v>9.713119000000006</v>
+      </c>
+      <c r="AB33">
+        <v>0.03796601284689501</v>
+      </c>
+      <c r="AC33">
+        <v>24.50676532703094</v>
+      </c>
     </row>
-    <row r="34" spans="1:23">
+    <row r="34" spans="1:29">
       <c r="A34" s="1">
         <v>46068.56431409722</v>
       </c>
@@ -2831,14 +3362,29 @@
       <c r="U34">
         <v>644.5488906540105</v>
       </c>
-      <c r="V34">
-        <v>1.229161418575824</v>
-      </c>
-      <c r="W34" t="b">
+      <c r="V34" t="b">
         <v>1</v>
       </c>
+      <c r="X34">
+        <v>0.241655216</v>
+      </c>
+      <c r="Y34">
+        <v>0.261077334</v>
+      </c>
+      <c r="Z34">
+        <v>0.3557507803906468</v>
+      </c>
+      <c r="AA34">
+        <v>9.711058999999999</v>
+      </c>
+      <c r="AB34">
+        <v>0.03797392009553861</v>
+      </c>
+      <c r="AC34">
+        <v>24.47604807136345</v>
+      </c>
     </row>
-    <row r="35" spans="1:23">
+    <row r="35" spans="1:29">
       <c r="A35" s="1">
         <v>46068.56443041666</v>
       </c>
@@ -2902,14 +3448,29 @@
       <c r="U35">
         <v>640.1619866851076</v>
       </c>
-      <c r="V35">
-        <v>2.844467989925458</v>
-      </c>
-      <c r="W35" t="b">
+      <c r="V35" t="b">
         <v>1</v>
       </c>
+      <c r="X35">
+        <v>0.2416714</v>
+      </c>
+      <c r="Y35">
+        <v>0.261082744</v>
+      </c>
+      <c r="Z35">
+        <v>0.3557657442651407</v>
+      </c>
+      <c r="AA35">
+        <v>9.705672</v>
+      </c>
+      <c r="AB35">
+        <v>0.03799502315727601</v>
+      </c>
+      <c r="AC35">
+        <v>24.32296950850848</v>
+      </c>
     </row>
-    <row r="36" spans="1:23">
+    <row r="36" spans="1:29">
       <c r="A36" s="1">
         <v>46068.56454615741</v>
       </c>
@@ -2973,11 +3534,26 @@
       <c r="U36">
         <v>644.0322268203383</v>
       </c>
-      <c r="V36">
-        <v>2.397589993227976</v>
-      </c>
-      <c r="W36" t="b">
+      <c r="V36" t="b">
         <v>1</v>
+      </c>
+      <c r="X36">
+        <v>0.241671718</v>
+      </c>
+      <c r="Y36">
+        <v>0.261077016</v>
+      </c>
+      <c r="Z36">
+        <v>0.3557617567481583</v>
+      </c>
+      <c r="AA36">
+        <v>9.702649000000001</v>
+      </c>
+      <c r="AB36">
+        <v>0.03800564466805986</v>
+      </c>
+      <c r="AC36">
+        <v>24.47685996731311</v>
       </c>
     </row>
   </sheetData>

</xml_diff>